<commit_message>
updated reasons sheet with boot details
</commit_message>
<xml_diff>
--- a/cmpe283/assignment3/reasons sheet.xlsx
+++ b/cmpe283/assignment3/reasons sheet.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/varunalla/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB903786-B9AF-F846-B16D-DD900C60A2CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{311F13F3-2CDC-B84A-AA21-38D553D518BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16400" xr2:uid="{28AD54D3-3234-E546-AFCA-7DDD04FE7BB8}"/>
+    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16400" activeTab="1" xr2:uid="{28AD54D3-3234-E546-AFCA-7DDD04FE7BB8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="exit reasons" sheetId="1" r:id="rId1"/>
+    <sheet name="firstcallpostboot" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -35,190 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
-  <si>
-    <t>CPUID(0x4ffffffc) 0:1377824</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 1:3166804</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 2:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 3:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 4:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) 7:3148562</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 8:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 9:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 10:214217184</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) 12:47492656</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 13:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 14:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 15:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 16:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) 18:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 19:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 20:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 21:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 22:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 23:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 24:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 25:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 26:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 27:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 28:600078492</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 29:69118</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 30:2639703966</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 31:4102812</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 32:383439504</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 33:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 34:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) 36:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 37:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) 39:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 40:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 41:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) 43:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 44:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 45:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 46:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 47:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 48:545934466</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 49:2339057058</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 50:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 51:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 52:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 53:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 54:29318</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 55:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 56:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 57:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 58:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 59:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 60:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 61:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 62:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 63:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 64:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) 67:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) 68:0</t>
-  </si>
-  <si>
-    <t>CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) CPUID(0x4ffffffc) 74:0</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="2">
   <si>
     <t>reason</t>
   </si>
@@ -587,10 +404,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>62</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -1091,315 +908,509 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2C17411-41DC-F645-9993-4282C6AE0D3C}">
-  <dimension ref="A1:A61"/>
+  <dimension ref="A1:B62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>30</v>
+      </c>
+      <c r="B2">
+        <v>730040</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>28</v>
+      </c>
+      <c r="B3">
+        <v>449125</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>227622</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
+        <v>49</v>
+      </c>
+      <c r="B5">
+        <v>169937</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
+        <v>32</v>
+      </c>
+      <c r="B6">
+        <v>66995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="1">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>47686</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="1">
+        <v>1</v>
+      </c>
+      <c r="B8">
+        <v>14843</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>48</v>
+      </c>
+      <c r="B9">
+        <v>11147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>6871</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>31</v>
+      </c>
+      <c r="B11">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>54</v>
+      </c>
+      <c r="B12">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="1">
+        <v>0</v>
+      </c>
+      <c r="B13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="1">
+        <v>29</v>
+      </c>
+      <c r="B14">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="B15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="1">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="B16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="1">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+      <c r="B17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="1">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="B18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="1">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+      <c r="B19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+      <c r="B20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+      <c r="B21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+      <c r="B22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+      <c r="B23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="B24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="1">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+      <c r="B25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+      <c r="B26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+      <c r="B27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+      <c r="B28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+      <c r="B29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+      <c r="B30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="1">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+      <c r="B31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="1">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+      <c r="B32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="1">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
+      <c r="B33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="1">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
+      <c r="B34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="1">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
+      <c r="B35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="1">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A38" t="s">
+      <c r="B36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="1">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
+      <c r="B37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="1">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
+      <c r="B38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="1">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A42" t="s">
+      <c r="B39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
         <v>41</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+      <c r="B40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
         <v>43</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+      <c r="B41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
         <v>44</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+      <c r="B42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
         <v>45</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+      <c r="B43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
         <v>46</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+      <c r="B44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
         <v>47</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+      <c r="B45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
         <v>50</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
+      <c r="B46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
         <v>51</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
+      <c r="B47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
         <v>52</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A54" t="s">
+      <c r="B48">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
         <v>53</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A55" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A56" t="s">
+      <c r="B49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
         <v>55</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A57" t="s">
+      <c r="B50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="1">
         <v>56</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
+      <c r="B51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="1">
         <v>57</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
+      <c r="B52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="1">
         <v>58</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
+      <c r="B53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="1">
         <v>59</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A61" t="s">
+      <c r="B54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="1">
         <v>60</v>
       </c>
+      <c r="B55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="1">
+        <v>61</v>
+      </c>
+      <c r="B56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="1">
+        <v>62</v>
+      </c>
+      <c r="B57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="1">
+        <v>63</v>
+      </c>
+      <c r="B58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="1">
+        <v>64</v>
+      </c>
+      <c r="B59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="1">
+        <v>67</v>
+      </c>
+      <c r="B60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="1">
+        <v>68</v>
+      </c>
+      <c r="B61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="1">
+        <v>74</v>
+      </c>
+      <c r="B62">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B63">
+    <sortCondition descending="1" ref="B2:B63"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>